<commit_message>
Fixes om een 8 te scoren.
</commit_message>
<xml_diff>
--- a/WEBFS - Nieuwe Functionaliteit v2.xlsx
+++ b/WEBFS - Nieuwe Functionaliteit v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stefan van Dockum\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cody.boelens\Desktop\WebFS_CodyBoelens_2192254\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73E099C-7D05-476E-A1CC-70602450BB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{038A31D7-34EC-489A-AADF-EFD466620E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A38A4BB1-9162-492B-8B56-A27CB18BE720}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{A38A4BB1-9162-492B-8B56-A27CB18BE720}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -406,13 +406,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF595959"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -445,7 +445,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -454,66 +454,93 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -535,9 +562,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -575,7 +602,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -681,7 +708,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -823,7 +850,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -832,596 +859,679 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC343CE-3199-4540-BCCF-A60B357088AA}">
   <dimension ref="A1:I79"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="57.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="84.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="6"/>
-    <col min="6" max="6" width="13.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" style="1"/>
-    <col min="9" max="9" width="23.42578125" style="12" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="37.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="57.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="84.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" style="3"/>
+    <col min="6" max="6" width="13.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="1"/>
+    <col min="9" max="9" width="23.44140625" style="4" customWidth="1"/>
+    <col min="10" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="14"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="1" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="11" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="I1" s="15"/>
+    </row>
+    <row r="2" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="6"/>
-      <c r="G3" s="3" t="s">
+      <c r="E2" s="16"/>
+      <c r="I2" s="15"/>
+    </row>
+    <row r="3" spans="1:9" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="G3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="13"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="H3" s="17"/>
+      <c r="I3" s="18"/>
+    </row>
+    <row r="4" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="13"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="6" t="s">
+      <c r="E4" s="29"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="31"/>
+    </row>
+    <row r="5" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="13"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C6" s="6" t="s">
+      <c r="E5" s="29"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="31"/>
+    </row>
+    <row r="6" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="13"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C7" s="6" t="s">
+      <c r="E6" s="29"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="31"/>
+    </row>
+    <row r="7" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="13"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="6" t="s">
+      <c r="E7" s="29"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="31"/>
+    </row>
+    <row r="8" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="13"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C9" s="6"/>
-      <c r="D9" s="7" t="s">
+      <c r="E8" s="29"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="31"/>
+    </row>
+    <row r="9" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="16"/>
+      <c r="D9" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="19" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="6"/>
-      <c r="D10" s="22" t="s">
+      <c r="I9" s="15"/>
+    </row>
+    <row r="10" spans="1:9" s="11" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="16"/>
+      <c r="D10" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-    </row>
-    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+    </row>
+    <row r="11" spans="1:9" s="11" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="25" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" s="19" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="I11" s="15"/>
+    </row>
+    <row r="12" spans="1:9" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="8">
         <v>5</v>
       </c>
-      <c r="I12" s="20"/>
-    </row>
-    <row r="13" spans="1:9" s="19" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="B13" s="16" t="s">
+      <c r="I12" s="9"/>
+    </row>
+    <row r="13" spans="1:9" s="11" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B13" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="27">
         <v>7</v>
       </c>
-      <c r="I13" s="20"/>
-    </row>
-    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
+      <c r="I13" s="15"/>
+    </row>
+    <row r="14" spans="1:9" s="11" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B14" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="27">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
+      <c r="I14" s="15"/>
+    </row>
+    <row r="15" spans="1:9" s="11" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="B15" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="27">
         <v>4</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
+      <c r="I15" s="15"/>
+    </row>
+    <row r="16" spans="1:9" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B16" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="8">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
+      <c r="I16" s="9"/>
+    </row>
+    <row r="17" spans="1:9" s="11" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B17" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="27">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B18" s="4" t="s">
+      <c r="I17" s="15"/>
+    </row>
+    <row r="18" spans="1:9" s="11" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="21">
+      <c r="E18" s="27">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="4" t="s">
+      <c r="I18" s="15"/>
+    </row>
+    <row r="19" spans="1:9" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B19" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="27">
         <v>10</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" s="19" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="I19" s="15"/>
+    </row>
+    <row r="20" spans="1:9" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="8">
         <v>4</v>
       </c>
-      <c r="I20" s="20"/>
-    </row>
-    <row r="21" spans="1:9" s="19" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="B21" s="16" t="s">
+      <c r="I20" s="9"/>
+    </row>
+    <row r="21" spans="1:9" s="5" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="B21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E21" s="21">
+      <c r="E21" s="8">
         <v>3</v>
       </c>
-      <c r="I21" s="20"/>
-    </row>
-    <row r="22" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
+      <c r="I21" s="9"/>
+    </row>
+    <row r="22" spans="1:9" s="11" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B22" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="27">
         <v>4</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="B23" s="4" t="s">
+      <c r="I22" s="15"/>
+    </row>
+    <row r="23" spans="1:9" s="11" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="B23" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="E23" s="21">
+      <c r="E23" s="27">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="B24" s="4"/>
-      <c r="C24" s="2"/>
-      <c r="E24" s="21"/>
-    </row>
-    <row r="25" spans="1:9" ht="270" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="I23" s="15"/>
+    </row>
+    <row r="24" spans="1:9" s="11" customFormat="1" ht="21" x14ac:dyDescent="0.3">
+      <c r="B24" s="12"/>
+      <c r="C24" s="26"/>
+      <c r="E24" s="27"/>
+      <c r="I24" s="15"/>
+    </row>
+    <row r="25" spans="1:9" s="5" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E25" s="21">
+      <c r="E25" s="8">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B26" s="4" t="s">
+      <c r="I25" s="9"/>
+    </row>
+    <row r="26" spans="1:9" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B26" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E26" s="21">
+      <c r="E26" s="8">
         <v>4</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B27" s="4" t="s">
+      <c r="I26" s="9"/>
+    </row>
+    <row r="27" spans="1:9" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E27" s="21">
+      <c r="E27" s="8">
         <v>4</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" s="19" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="B28" s="16" t="s">
+      <c r="I27" s="9"/>
+    </row>
+    <row r="28" spans="1:9" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E28" s="21">
+      <c r="E28" s="8">
         <v>4</v>
       </c>
-      <c r="I28" s="20"/>
-    </row>
-    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B29" s="4"/>
-      <c r="C29" s="2" t="s">
+      <c r="I28" s="9"/>
+    </row>
+    <row r="29" spans="1:9" s="5" customFormat="1" ht="21" x14ac:dyDescent="0.3">
+      <c r="B29" s="6"/>
+      <c r="C29" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E29" s="21">
+      <c r="E29" s="8">
         <v>7</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="B30" s="4"/>
-      <c r="C30" s="2"/>
-      <c r="E30" s="21"/>
-    </row>
-    <row r="31" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="I29" s="9"/>
+    </row>
+    <row r="30" spans="1:9" s="11" customFormat="1" ht="21" x14ac:dyDescent="0.3">
+      <c r="B30" s="12"/>
+      <c r="C30" s="26"/>
+      <c r="E30" s="27"/>
+      <c r="I30" s="15"/>
+    </row>
+    <row r="31" spans="1:9" s="11" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="E31" s="21">
+      <c r="E31" s="27">
         <v>11</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" s="19" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="B32" s="16" t="s">
+      <c r="I31" s="15"/>
+    </row>
+    <row r="32" spans="1:9" s="11" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B32" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="E32" s="21">
+      <c r="E32" s="27">
         <v>11</v>
       </c>
-      <c r="I32" s="20"/>
-    </row>
-    <row r="33" spans="2:9" ht="195" x14ac:dyDescent="0.25">
-      <c r="B33" s="4" t="s">
+      <c r="I32" s="15"/>
+    </row>
+    <row r="33" spans="2:9" s="5" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="B33" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E33" s="21">
+      <c r="E33" s="8">
         <v>8</v>
       </c>
-      <c r="I33" s="1"/>
-    </row>
-    <row r="34" spans="2:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="B34" s="4" t="s">
+    </row>
+    <row r="34" spans="2:9" s="5" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="B34" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E34" s="21">
+      <c r="E34" s="8">
         <v>6</v>
       </c>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C35" s="2"/>
-      <c r="E35" s="6">
+      <c r="I34" s="9"/>
+    </row>
+    <row r="35" spans="2:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C35" s="26"/>
+      <c r="E35" s="16">
         <f>SUM(E12:E34)</f>
         <v>130</v>
       </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I35" s="15"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C36" s="2"/>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C37" s="2"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C38" s="2"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C39" s="2"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C40" s="2"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C41" s="2"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C42" s="2"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C43" s="2"/>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C37" s="7"/>
+      <c r="E37" s="10"/>
+      <c r="I37" s="9"/>
+    </row>
+    <row r="38" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C38" s="7"/>
+      <c r="E38" s="10"/>
+      <c r="I38" s="9"/>
+    </row>
+    <row r="39" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C39" s="7"/>
+      <c r="E39" s="10"/>
+      <c r="I39" s="9"/>
+    </row>
+    <row r="40" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C40" s="7"/>
+      <c r="E40" s="10"/>
+      <c r="I40" s="9"/>
+    </row>
+    <row r="41" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C41" s="7"/>
+      <c r="E41" s="10"/>
+      <c r="I41" s="9"/>
+    </row>
+    <row r="42" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C42" s="7"/>
+      <c r="E42" s="10"/>
+      <c r="I42" s="9"/>
+    </row>
+    <row r="43" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C43" s="7"/>
+      <c r="E43" s="10"/>
+      <c r="I43" s="9"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="2"/>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C46" s="2"/>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C47" s="2"/>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C48" s="2"/>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C49" s="2"/>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C50" s="2"/>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C51" s="2"/>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C52" s="2"/>
-    </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C53" s="2"/>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C54" s="2"/>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C55" s="2"/>
-    </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C56" s="2"/>
-    </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C57" s="2"/>
-    </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C58" s="2"/>
-    </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C59" s="2"/>
-    </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C60" s="2"/>
-    </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C61" s="2"/>
-    </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C49" s="7"/>
+      <c r="E49" s="10"/>
+      <c r="I49" s="9"/>
+    </row>
+    <row r="50" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C50" s="7"/>
+      <c r="E50" s="10"/>
+      <c r="I50" s="9"/>
+    </row>
+    <row r="51" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C51" s="7"/>
+      <c r="E51" s="10"/>
+      <c r="I51" s="9"/>
+    </row>
+    <row r="52" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C52" s="7"/>
+      <c r="E52" s="10"/>
+      <c r="I52" s="9"/>
+    </row>
+    <row r="53" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C53" s="7"/>
+      <c r="E53" s="10"/>
+      <c r="I53" s="9"/>
+    </row>
+    <row r="54" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C54" s="7"/>
+      <c r="E54" s="10"/>
+      <c r="I54" s="9"/>
+    </row>
+    <row r="55" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C55" s="7"/>
+      <c r="E55" s="10"/>
+      <c r="I55" s="9"/>
+    </row>
+    <row r="56" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C56" s="7"/>
+      <c r="E56" s="10"/>
+      <c r="I56" s="9"/>
+    </row>
+    <row r="57" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C57" s="7"/>
+      <c r="E57" s="10"/>
+      <c r="I57" s="9"/>
+    </row>
+    <row r="58" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C58" s="7"/>
+      <c r="E58" s="10"/>
+      <c r="I58" s="9"/>
+    </row>
+    <row r="59" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C59" s="7"/>
+      <c r="E59" s="10"/>
+      <c r="I59" s="9"/>
+    </row>
+    <row r="60" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="7"/>
+      <c r="E60" s="10"/>
+      <c r="I60" s="9"/>
+    </row>
+    <row r="61" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="7"/>
+      <c r="E61" s="10"/>
+      <c r="I61" s="9"/>
+    </row>
+    <row r="62" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C62" s="2"/>
     </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C63" s="2"/>
     </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C64" s="2"/>
     </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="2"/>
-    </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="2"/>
-    </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C67" s="2"/>
-    </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="2"/>
-    </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C69" s="2"/>
-    </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="2"/>
-    </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C71" s="2"/>
-    </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C72" s="2"/>
-    </row>
-    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C65" s="7"/>
+      <c r="E65" s="10"/>
+      <c r="I65" s="9"/>
+    </row>
+    <row r="66" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C66" s="7"/>
+      <c r="E66" s="10"/>
+      <c r="I66" s="9"/>
+    </row>
+    <row r="67" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C67" s="7"/>
+      <c r="E67" s="10"/>
+      <c r="I67" s="9"/>
+    </row>
+    <row r="68" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C68" s="7"/>
+      <c r="E68" s="10"/>
+      <c r="I68" s="9"/>
+    </row>
+    <row r="69" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C69" s="7"/>
+      <c r="E69" s="10"/>
+      <c r="I69" s="9"/>
+    </row>
+    <row r="70" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C70" s="7"/>
+      <c r="E70" s="10"/>
+      <c r="I70" s="9"/>
+    </row>
+    <row r="71" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C71" s="7"/>
+      <c r="E71" s="10"/>
+      <c r="I71" s="9"/>
+    </row>
+    <row r="72" spans="3:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C72" s="7"/>
+      <c r="E72" s="10"/>
+      <c r="I72" s="9"/>
+    </row>
+    <row r="73" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C73" s="2"/>
     </row>
-    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C74" s="2"/>
     </row>
-    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C75" s="2"/>
     </row>
-    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C76" s="2"/>
     </row>
-    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C77" s="2"/>
     </row>
-    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C78" s="2"/>
     </row>
-    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C79" s="2"/>
     </row>
   </sheetData>

</xml_diff>